<commit_message>
One Migration, Start to Finish: the eight stages walked through on a single engagement
</commit_message>
<xml_diff>
--- a/guides/data-migration-stages/toolkit/Migration-Gate-Sign-off-Sheet.xlsx
+++ b/guides/data-migration-stages/toolkit/Migration-Gate-Sign-off-Sheet.xlsx
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="F2" s="9" t="n">
-        <v>46094</v>
+        <v>46101</v>
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="F3" s="9" t="n">
-        <v>46108</v>
+        <v>46120</v>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
@@ -1117,7 +1117,7 @@
         </is>
       </c>
       <c r="F4" s="9" t="n">
-        <v>46136</v>
+        <v>46150</v>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>46153</v>
+        <v>46181</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -1197,7 +1197,7 @@
         </is>
       </c>
       <c r="F6" s="9" t="n">
-        <v>46162</v>
+        <v>46203</v>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="F7" s="9" t="n">
-        <v>46176</v>
+        <v>46223</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
@@ -1266,27 +1266,21 @@
           <t>Go-live accepted</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>A. Reyes</t>
-        </is>
-      </c>
+      <c r="D8" s="7" t="inlineStr"/>
       <c r="E8" s="7" t="inlineStr">
         <is>
           <t>Client PM</t>
         </is>
       </c>
-      <c r="F8" s="9" t="n">
-        <v>46185</v>
-      </c>
+      <c r="F8" s="7" t="n"/>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Post-load reconciliation, every row Pass</t>
+          <t>Pending. Post-load reconciliation runs to 03 August.</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Signed</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1309,7 @@
       <c r="F9" s="7" t="n"/>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Pending. Hypercare window ends 10 July.</t>
+          <t>Pending. Hypercare closes 03 September.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">

</xml_diff>